<commit_message>
Cập nhật danh sách tài khoản ngày 20/5/2026
Cập nhật danh sách tài khoản ngày 20/5/2026
</commit_message>
<xml_diff>
--- a/docs/testdata/Danhsachtaikhoan.xlsx
+++ b/docs/testdata/Danhsachtaikhoan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BTL\Kì 8\DATN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40952667-9A5B-403A-A104-5279EC5D8599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA5E587A-1F1E-46E9-B09A-17C9CDBAB922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2A474757-1352-4CA6-BD0B-51A09DEC4E77}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="70">
   <si>
     <t xml:space="preserve">Bảng tài khoản </t>
   </si>
@@ -156,6 +156,104 @@
   </si>
   <si>
     <t xml:space="preserve">Ngày tạo  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Reset Iphone
+2.  Kết nối 4G để tải app
+3. Tải qua tool ảo 
+4. Ko kết nối wifi khi tạo tài khoản
+5. Thuê số đt  web dvdd
+add mail, sử dụng tài khoản như  người thật trong vòng 10p </t>
+  </si>
+  <si>
+    <t>Testshopee01@</t>
+  </si>
+  <si>
+    <t>x5sfnlupa2</t>
+  </si>
+  <si>
+    <t>SPC_ST=c3Rma0ZQYXR5MkpEWEt0di7YmSK9FD0nxPZOenRrsA1/6Alz1pgUC/dfEbilkEGLKMGi3P4OSiByYZhPcSARS2iZW8aNnRC8MqzzhJSxiIysxD0OFDdw5a5twq48NYRKUgs4DpiCpDb2JfCXXFtQSePwJx9jcugYfrjjmLO6bQSdD/zIqw2PbGE8/OgP4a8Y+OTK0iVq6dwGLRZszraIuA==.ALwMVKjGBLS7Bhxj9j91oAjLgtro98HGZp/GAdzS7l4p</t>
+  </si>
+  <si>
+    <t>wessonpriceonhl@outlook.com|5pWHZ8nggr|M.C553_BL2.0.U.-CnhqSXH7QkW40JnlChwtaY1fEkS02ZHC0PkyFdokXdSp4Re073dXAiTu!BIWaSYDsv!aCWYm1Oan6d1wBy*08HKBQqumyr5TWaWDMT*J0wsRvptcW314qRMthUdMgVwOHqW0liVgFSbSZsz1Yp9letlfosdv!MbS88L7kFZCkzPvCsXTq7sTSM!g7mJUwyiQ7sIpNWsPUVIArsvcc7ozxIc8yZ8!JMG01KTIVQ5RXY*HWZAKxLFAf7*q5*gVq5P5KymLAA0wKYdtwn7c5OZJaedWz8TSJ9XXATldDoRAfccXFUDpl*VGpbMpfHbvO0HT6tAXJelQ6K3VMmM0LhMPojbkbcG!rjUT7CVNdvA5gSXCeJFguWUDLMQCeIhcTfbO9S54X8A0Y7klM6TB1CCvNwliGyWczhtpgtyt!7v99iCG|9e5f94bc-e8a4-4e73-b8be-63364c29d753</t>
+  </si>
+  <si>
+    <t>Motest99@</t>
+  </si>
+  <si>
+    <t>o0jbjaklcx</t>
+  </si>
+  <si>
+    <t>SPC_ST=QWdvbTduNGl4RjdLbnV6aHkzxkjQfAQ7k6ku7xbZrM8x2q7+rTDNaQt3rLULfBocHgeZFlLKMK5Yeq+w2v3nz3CyyV5Rmk3t+na5accpBwKWV72HmcpQ8gQFmV3x/9NTtiNQf51B2OAiOa9Cn8X7TXRTySi7XO33aerQckeMB32eTiBAPtaI6ld8C2RHqiE5.AIJrgvy4RvXgEZ8nui3MaBEsMwJ2rB1IzJE3fQ+dstZN</t>
+  </si>
+  <si>
+    <t>zavierstoutyymy@outlook.com|PTMsEtHT9m|M.C502_BL2.0.U.-CsK!8p5NTjpbURQHUrpdhc9I36m*cGtU81CJ0fg4PUbadvPKufhR7etvKtsXAsDmm9vjOS54VO950IkmRBySM6Us!Cd8QGMU6oPBYR18XGPUTz5eEah4JMsXgK6MTCRRW045e2bT3JHEqpdXCvzp36E8tpx1cvzxzUaJOU8oNY5HCsoOqVxV!8VSlvsegxKgLvMHlZatLIXyshXh*w!euT392l49q67FpPbffZOvphL00KTRKY534Y050HI!I0G3eX3cT9nxXHZdL3d4ziiIDTed*8KzNPvl3R0tn7pDopKPRC4OmRs!85Cdkms9A4XZ194mHD*A1j1mlz1Se5W6AKUxMxeL7lzQpf7NsKnpWKraysOUhUzgeqNHbzFNd3rc2ZPz7awmXPm9xwA6HmxuXLZ8TIWUnLDD55UZYzg*r4tB|9e5f94bc-e8a4-4e73-b8be-63364c29d753</t>
+  </si>
+  <si>
+    <t>Tài khoản vừa tạo thì bị lỗi trang không khả dụng</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>acb1bmi9se</t>
+  </si>
+  <si>
+    <t>9zx_gxsebf</t>
+  </si>
+  <si>
+    <t>9qhke012p5</t>
+  </si>
+  <si>
+    <t>98wyhm2138</t>
+  </si>
+  <si>
+    <t>8np5jlrbq2</t>
+  </si>
+  <si>
+    <t>Lhvo6mm68</t>
+  </si>
+  <si>
+    <t>Pnnjdmg72</t>
+  </si>
+  <si>
+    <t>Py7o5jx84</t>
+  </si>
+  <si>
+    <t>Y35fo7917</t>
+  </si>
+  <si>
+    <t>Eme9d3h06</t>
+  </si>
+  <si>
+    <t>.shopee.vn=SPC_F=Almzl7t2qFJqlYD31Age1gBPZRJkD0YJ</t>
+  </si>
+  <si>
+    <t>.shopee.vn=SPC_F=23FDGIuiLu9XCBDJyQGALOaageAZxp1z</t>
+  </si>
+  <si>
+    <t>.shopee.vn=SPC_F=fSW4Z2DaqKnuVR0lMJQ39aT3GgOqd6jI</t>
+  </si>
+  <si>
+    <t>.shopee.vn=SPC_F=xekuunIA6Y0Qvyk3AXri5wFpKLeT97hL</t>
+  </si>
+  <si>
+    <t>.shopee.vn=SPC_F=0aNP8p6A0ZEDbrOMswmWvoXcjexb3sep</t>
+  </si>
+  <si>
+    <t>marshallrobertsononin@outlook.com|tSumDa6nxs|M.C510_SN1.0.U.-Cqi5CeGd3xTRykjSQEOOwOHARyE*TdCpop7aeIRNkjy029UKR8jlYm3qRhdyMzE2N8QsaS2EPa9fmHjadT!SiAfxcMsnGxnaiyJc9mZGnudlWCeeSjfBEV4SPvRfV3Gi2DyLzXtJREWgIoa*dOvs*ONTbVK63s5re!XbuCI9IRdHxrSf0rCXTrXdAq0tZu*ty0is8CchqJ2tLfCQHxEpTG6CflLfuQWN*pOHrD3VFDsgLzgsU2B8lspfmRikrmQFYworQ*qEO2qxVZHpXOhwRcKqDliFf4Hh!MxIbBse0c*CMrhCdrj0CeSLmOpoPRIHK3TCm7q*49klYTHKGPwVxBZ1SKhX491eq!PrFsosNcx2HCAFk7PgrWfsMd6LTQpb7krLUEWmX2MKLgwAiXcP*bJW6tKpAFxn4waUn!OyFotvLwnTppiOsZrgW8vLNBVBSw$$|9e5f94bc-e8a4-4e73-b8be-63364c29d753</t>
+  </si>
+  <si>
+    <t>nikolasmathewshogt@outlook.com|J3PYVdRbfz|M.C545_BAY.0.U.-CklOZLFHQL3sZ5mJjtVGY**4IYLBO!zGOFA4WWLLXUqT2IcEVcL2WDNKiwZAH*Gp5xhXXXlh7YbFmzpWJXqHC74tUVhFohxMjStrAQlLW*zm1ovoG69LP*w6DcPTWv1IkOF04RvPtwyR0MVIFRwWhzUOdanWtvRw2j9Wuo9Xpel3PsobfTyuhksxrUSD1UhVmQQa8N4dt0cooZ9F13GqOT*Q6rAUvs2awK!o1YQb1c3haT0r4LhqAv4MzCb7WVh*Uyl3e!Yvzf0dEd2QdAznPzW2oME15OO4h0opGYvVm34mcXQJhr7cIEG1AMTOdDOfIkoIEn2ov2iE05CCvPKV1J3MeEyMafw00WoQ2QD0i1mw9rqRix5sBnHnpr2Anu2Ba9RaZQ6Jc9DdGZrZpN1zMtg4xmXPoFP6YkrpGy7W1POKpRHHYXGXDCNqTnFg8JqvWQ$$|9e5f94bc-e8a4-4e73-b8be-63364c29d753</t>
+  </si>
+  <si>
+    <t>dakarihendersongtyu@outlook.com|P8hvkSeavh|M.C508_BAY.0.U.-ClVeUAqaDVdFDisHqwHB6mfj5QnPwKFn30HHHCR!PSqMX4BETydSdfpW4ukEmq78Ta1lpa4qWHVRedhoQyxsQd85r*m0ZOcsbaboqJxXYXkOfj*nmUbicVcpaUApdkvsBxTem*0pq1ScNdrzkyqyZP2oCWhQqZddkXZ*JeXDBEdpwBMI1sEupW!8hqNesND3QbuRfEOocWKJGNwYXoj3EWVxH00U43*iVuzRbUJIkgSpPEaqZRIHFqs3mMfWEIOOCjF1XIitYsdGpVsOMnFG2awpOGt2SGZPdHIPJIs7KDY9fHdDF*gETAk4AoFoPqCyeENSFX2Xnxmxx2rpRXrnbNkL!G!BIyNFjezhiac*4YlBYwCLwcJ57uhAOoyHNa*5HKFFcPQ8cru19I9nAv7EnVOv1hmkAtCMv01iUEE7ZeBq|9e5f94bc-e8a4-4e73-b8be-63364c29d753</t>
+  </si>
+  <si>
+    <t>augustusnortoncmjw@outlook.com|UBKt4Wco1Q|M.C525_BAY.0.U.-Cv29HbLpga1twhmuvjUUrkj14xEX9HmUFGYm5Aweyy4g1vSwnq*H5LhmJnlW3b5RUebFjSVtycn0uVKh3e32s!ZWnS1fcrFJKIRJXobdBhga7ouSZ21qfyHdd1UCHoYtu1FY!mm1GKmkmu77qakQ9ezR5!BO59RcSjSEJla84Djf*m8NtyngsVTvs0*WFFrXOOK8Nlezh91s59LKuffkOnp8Djs60nNrENbcKWYAcRTNW2!NLE6YVttSA!9W!swFqIGxhwc9x*ZWG!NZCovIacukuYwEFeH853G2wc*o0SfZ*zXRPNb06wQIXWQTtOMoxUiQUdF7FUJDLhm6m6aPn!gnwHE3bROQHmq8klDL76!ApxM*GofqMSxH58PGPW4qxVi8k2u6CtMbmtMZ1jeXcnxPnBb0ap2YCoCUIRUQ7kuD|9e5f94bc-e8a4-4e73-b8be-63364c29d753</t>
+  </si>
+  <si>
+    <t>lianwatershzoi@outlook.com|ildDP6MF7g|M.C523_SN1.0.U.-Ctst9cUewLnMc97MUaF2fe7g14jD6EGb6pNGpSPVLO8WCtd6DjSdiwSI6H4AcV3oCCRSk7kU5KpDY3Qko28uDDpx5T9LBW2Zqe40E8*DxoTG2MmFtwRAllKnocb8nicLD1ofI0RuWG6du50iKEL2d49S!mga1nBfhJWe7odNjFT9oPydF7QeeED1KTxq5MufCZpclhOmtYBcLMzEBsuC1TVjx3835ygx*YlsPvUEWmAhp0DIt2lcI1GR!th2c7mmjBP!FAW882N0bGxcX94V9X9kf9Hr*vyy67vOXROy7H2Kq7bC9O5YoIeswGcFcZ8csxKyxPNzuuCSk6szsHTFsUgCvAb6Sz5TYHR!E1hiNUpQvDnhxdHZ2tvKarwgCwhkJDsT4feIMPQKJ9Baq3R952BVxNVDDT97aW9EpKpQ1Cb1|9e5f94bc-e8a4-4e73-b8be-63364c29d753</t>
   </si>
 </sst>
 </file>
@@ -221,7 +319,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -290,27 +388,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -318,12 +444,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -333,10 +464,44 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -355,14 +520,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFCCC0D9"/>
-          <bgColor rgb="FFCCC0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFC2D69B"/>
           <bgColor rgb="FFC2D69B"/>
         </patternFill>
@@ -373,6 +530,14 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFEA5444"/>
           <bgColor rgb="FFEA5444"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCCC0D9"/>
+          <bgColor rgb="FFCCC0D9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -686,7 +851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22CF1B0D-0482-4E78-85C7-359723D6CFFB}">
-  <dimension ref="D2:S34"/>
+  <dimension ref="D2:N32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="3.6640625" customWidth="1"/>
@@ -696,67 +861,67 @@
     <col min="9" max="10" width="20.77734375" customWidth="1"/>
     <col min="11" max="11" width="36" customWidth="1"/>
     <col min="12" max="12" width="17.5546875" customWidth="1"/>
-    <col min="13" max="13" width="29.21875" style="6" customWidth="1"/>
+    <col min="13" max="13" width="29.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="4:19" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="D2" s="14" t="s">
+    <row r="2" spans="4:14" ht="19.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="16"/>
-    </row>
-    <row r="3" spans="4:19" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="17" t="s">
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="14"/>
+    </row>
+    <row r="3" spans="4:14" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="17" t="s">
+      <c r="G3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="17" t="s">
+      <c r="I3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="17" t="s">
+      <c r="J3" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="K3" s="17" t="s">
+      <c r="K3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="18" t="s">
+      <c r="L3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="17" t="s">
+      <c r="M3" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="N3" s="17" t="s">
+      <c r="N3" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="4:19" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="4:14" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D4" s="1">
         <v>1</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="10">
         <v>46161</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="1" t="s">
@@ -768,27 +933,27 @@
       <c r="I4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="3" t="s">
+      <c r="J4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L4" s="10" t="s">
+      <c r="L4" s="5" t="s">
         <v>20</v>
       </c>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
     </row>
-    <row r="5" spans="4:19" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="4:14" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D5" s="1">
         <v>2</v>
       </c>
-      <c r="E5" s="5"/>
-      <c r="F5" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" s="3" t="s">
+      <c r="E5" s="11"/>
+      <c r="F5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="H5" s="1" t="s">
@@ -797,258 +962,386 @@
       <c r="I5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J5" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="K5" s="3" t="s">
+      <c r="J5" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="10" t="s">
+      <c r="L5" s="5" t="s">
         <v>20</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
     </row>
-    <row r="6" spans="4:19" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="4:14" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D6" s="1">
         <v>3</v>
       </c>
-      <c r="E6" s="5"/>
-      <c r="F6" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="2" t="s">
+      <c r="E6" s="11"/>
+      <c r="F6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="K6" s="2" t="s">
+      <c r="J6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L6" s="10" t="s">
+      <c r="L6" s="5" t="s">
         <v>20</v>
       </c>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="6"/>
-    </row>
-    <row r="7" spans="4:19" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="4:14" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D7" s="1">
         <v>4</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="2" t="s">
+      <c r="E7" s="11"/>
+      <c r="F7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J7" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" s="3" t="s">
+      <c r="J7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="L7" s="10" t="s">
+      <c r="L7" s="5" t="s">
         <v>20</v>
       </c>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
-    </row>
-    <row r="8" spans="4:19" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="4:14" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D8" s="1">
         <v>5</v>
       </c>
-      <c r="E8" s="5"/>
-      <c r="F8" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="2" t="s">
+      <c r="E8" s="11"/>
+      <c r="F8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J8" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="K8" s="3" t="s">
+      <c r="J8" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="L8" s="5" t="s">
         <v>20</v>
       </c>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
-      <c r="Q8" s="6"/>
-      <c r="R8" s="6"/>
-      <c r="S8" s="6"/>
-    </row>
-    <row r="9" spans="4:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D9" s="2">
+    </row>
+    <row r="9" spans="4:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D9" s="1">
         <v>6</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="25">
         <v>46161</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="15">
         <v>522385216</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="I9" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="J9" s="1" t="s">
+      <c r="I9" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="K9" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="L9" s="10" t="s">
+      <c r="L9" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="M9" s="11" t="s">
+      <c r="M9" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="N9" s="1"/>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6"/>
-    </row>
-    <row r="10" spans="4:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M10"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="6"/>
-    </row>
-    <row r="11" spans="4:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M11"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-    </row>
-    <row r="12" spans="4:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="J12" s="12"/>
-      <c r="M12"/>
-    </row>
-    <row r="13" spans="4:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M13"/>
-    </row>
-    <row r="14" spans="4:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M14"/>
-    </row>
-    <row r="15" spans="4:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M15"/>
-    </row>
-    <row r="16" spans="4:19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M16"/>
-    </row>
-    <row r="17" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M17"/>
-    </row>
-    <row r="18" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M18"/>
-    </row>
-    <row r="19" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M19"/>
-    </row>
-    <row r="20" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M20"/>
-    </row>
-    <row r="21" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M21"/>
-    </row>
-    <row r="22" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M22"/>
-    </row>
-    <row r="23" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M23"/>
-    </row>
-    <row r="24" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M24"/>
-    </row>
-    <row r="25" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M25"/>
-    </row>
-    <row r="26" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M26"/>
-    </row>
-    <row r="27" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M27"/>
-    </row>
-    <row r="28" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M28"/>
-    </row>
-    <row r="29" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M29"/>
-    </row>
-    <row r="30" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M30"/>
-    </row>
-    <row r="31" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="L31" s="6"/>
-      <c r="M31"/>
-    </row>
-    <row r="32" spans="12:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="L32" s="6"/>
-      <c r="M32"/>
-    </row>
-    <row r="33" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L33" s="6"/>
-    </row>
-    <row r="34" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L34" s="6"/>
-    </row>
+      <c r="N9" s="15"/>
+    </row>
+    <row r="10" spans="4:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D10" s="15">
+        <v>7</v>
+      </c>
+      <c r="E10" s="26">
+        <v>46162</v>
+      </c>
+      <c r="F10" s="15">
+        <v>522392281</v>
+      </c>
+      <c r="G10" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="I10" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J10" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="K10" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="L10" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="M10" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N10" s="15"/>
+    </row>
+    <row r="11" spans="4:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D11" s="1">
+        <v>8</v>
+      </c>
+      <c r="E11" s="26">
+        <v>46162</v>
+      </c>
+      <c r="F11" s="1"/>
+      <c r="G11" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="I11" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="J11" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="L11" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="4:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D12" s="1">
+        <v>9</v>
+      </c>
+      <c r="E12" s="24">
+        <v>46162</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="I12" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="L12" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+    </row>
+    <row r="13" spans="4:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D13" s="1">
+        <v>10</v>
+      </c>
+      <c r="E13" s="30"/>
+      <c r="F13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="I13" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L13" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+    </row>
+    <row r="14" spans="4:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D14" s="1">
+        <v>11</v>
+      </c>
+      <c r="E14" s="30"/>
+      <c r="F14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I14" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="L14" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+    </row>
+    <row r="15" spans="4:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D15" s="1">
+        <v>12</v>
+      </c>
+      <c r="E15" s="30"/>
+      <c r="F15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="I15" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="L15" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+    </row>
+    <row r="16" spans="4:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D16" s="1">
+        <v>13</v>
+      </c>
+      <c r="E16" s="31"/>
+      <c r="F16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I16" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="L16" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+    </row>
+    <row r="17" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="20" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="21" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="22" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="23" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="24" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="25" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="26" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="27" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="28" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="29" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="30" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="31" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="32" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="E4:E8"/>
     <mergeCell ref="D2:N2"/>
+    <mergeCell ref="E12:E16"/>
   </mergeCells>
-  <conditionalFormatting sqref="L4:L9">
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="Failed">
+  <conditionalFormatting sqref="L4:L16">
+    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Accepted">
+      <formula>NOT(ISERROR(SEARCH(("Accepted"),(L4))))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH(("Failed"),(L4))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="Passed">
+    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="Passed">
       <formula>NOT(ISERROR(SEARCH(("Passed"),(L4))))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L9">
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Accepted">
-      <formula>NOT(ISERROR(SEARCH(("Accepted"),(L4))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L9">
     <cfRule type="containsText" dxfId="0" priority="6" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH(("Pending"),(L4))))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L9">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -1061,7 +1354,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L4:L9" xr:uid="{EBA59FE4-09DB-480F-A962-B3086650315B}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L4:L16" xr:uid="{EBA59FE4-09DB-480F-A962-B3086650315B}">
       <formula1>"Passed,Failed,Untested,Pending,Accepted,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1073,6 +1366,11 @@
     <hyperlink ref="K7" r:id="rId5" display="|quintontorresbcfm@outlook.com|ZfFo5T3N58|M.C524_SN1.0.U.-CjumdlUuma!qN6SR7lUlQBGoQS2RKNzLZtm!CBCpf9uYAk0NSrYDK5BYDBRI1*83B4SmMyYLxmkSCQM4VelDPeptFhY9U8r5KkTrO87jNCz1kPxqVZLC1yWQHeiHLjReaREh5oOe5shl6tn09S3tr!xoBa2cMZA0SpmBi75vfbX5uE0lonHoauxX6irDlcIK40hmY54T2dJmS1SQsiGlUxa55rNH0PPFvcR5sO*SprEC7qZI6oRCJghDVyEpIObIJyLGZrNzWUTEgX3ThQ05fe78Giq*!yJHuGmzdnDhW9ocGKjWUC0lpECIdtEL4SDEVSF7!3WR8iUjreXwoStPoVnLxh0Yf3LUfg1fCzCFbcoG*79SJuRP9TCCPuZoCX3LiXp9nHfRSqrmb0wifuG8k*DUHD7SX!CrM*w!Z4g!ACD*|9e5f94bc-e8a4-4e73-b8be-63364c29d753" xr:uid="{2180D885-B07D-4212-9A63-86244029C208}"/>
     <hyperlink ref="H9" r:id="rId6" xr:uid="{A182E084-0B68-4859-B972-0B6BFA2EA35B}"/>
     <hyperlink ref="K9" r:id="rId7" display="coltbradleydfwt@outlook.com|ltvyU67E1i|M.C533_SN1.0.U.-CuYFhmbD0vaMoK4LzrzFtSr5sI9fYMCyDAJvOeffM5c3ho6veSlSNigt4gKFLsR6QUDukjWZ2NpPE1jG1T5hBWb0LQponfctOo2IVQ4Rkx*qMHktweS8YGJLL32LLZAJBZv10Y10EZ32YbNCQLuWKaxdXoWjbaNAvqgMIeR5KW*lLcJGAvupEf7WADbniTkbwtdvAefCCqy7JMf4WiAIsZrfkwCKxWsh77piv2Z8cbeWZxH8Tgmtmr3g6QeeAAuAZzSL265Pfn7evrmztFJrHeQ0cRYvpwZrVO!W5UK9kDg!o!0wzlVC71lO9GWYKcuZ3vrniHrn4tSCv*rmLV*HsbpYcfExq1Ye5W8Lh6ErS3merVLsmMdlfe7rnJd1w7*SWEVtE7LZTA9ujiyl*qSxDNXaxwZnaW!ThoLWKxzJrD!r|9e5f94bc-e8a4-4e73-b8be-63364c29d753" xr:uid="{097FAE64-8E05-49F2-8BA1-CDAB6454B23E}"/>
+    <hyperlink ref="H10" r:id="rId8" xr:uid="{CB9F0AE6-2617-4A44-B751-1410D1FE092E}"/>
+    <hyperlink ref="H11" r:id="rId9" xr:uid="{478BBA64-C152-4D18-8B86-A3ACA082F3AC}"/>
+    <hyperlink ref="K13" r:id="rId10" display="marshallrobertsononin@outlook.com|tSumDa6nxs|M.C510_SN1.0.U.-Cqi5CeGd3xTRykjSQEOOwOHARyE*TdCpop7aeIRNkjy029UKR8jlYm3qRhdyMzE2N8QsaS2EPa9fmHjadT!SiAfxcMsnGxnaiyJc9mZGnudlWCeeSjfBEV4SPvRfV3Gi2DyLzXtJREWgIoa*dOvs*ONTbVK63s5re!XbuCI9IRdHxrSf0rCXTrXdAq0tZu*ty0is8CchqJ2tLfCQHxEpTG6CflLfuQWN*pOHrD3VFDsgLzgsU2B8lspfmRikrmQFYworQ*qEO2qxVZHpXOhwRcKqDliFf4Hh!MxIbBse0c*CMrhCdrj0CeSLmOpoPRIHK3TCm7q*49klYTHKGPwVxBZ1SKhX491eq!PrFsosNcx2HCAFk7PgrWfsMd6LTQpb7krLUEWmX2MKLgwAiXcP*bJW6tKpAFxn4waUn!OyFotvLwnTppiOsZrgW8vLNBVBSw$$|9e5f94bc-e8a4-4e73-b8be-63364c29d753" xr:uid="{5A4BA726-8EEF-420B-BF51-2185739ADAA2}"/>
+    <hyperlink ref="K14" r:id="rId11" display="dakarihendersongtyu@outlook.com|P8hvkSeavh|M.C508_BAY.0.U.-ClVeUAqaDVdFDisHqwHB6mfj5QnPwKFn30HHHCR!PSqMX4BETydSdfpW4ukEmq78Ta1lpa4qWHVRedhoQyxsQd85r*m0ZOcsbaboqJxXYXkOfj*nmUbicVcpaUApdkvsBxTem*0pq1ScNdrzkyqyZP2oCWhQqZddkXZ*JeXDBEdpwBMI1sEupW!8hqNesND3QbuRfEOocWKJGNwYXoj3EWVxH00U43*iVuzRbUJIkgSpPEaqZRIHFqs3mMfWEIOOCjF1XIitYsdGpVsOMnFG2awpOGt2SGZPdHIPJIs7KDY9fHdDF*gETAk4AoFoPqCyeENSFX2Xnxmxx2rpRXrnbNkL!G!BIyNFjezhiac*4YlBYwCLwcJ57uhAOoyHNa*5HKFFcPQ8cru19I9nAv7EnVOv1hmkAtCMv01iUEE7ZeBq|9e5f94bc-e8a4-4e73-b8be-63364c29d753" xr:uid="{AADDA024-CE6F-4486-88FE-F2C762815D2D}"/>
+    <hyperlink ref="K16" r:id="rId12" display="augustusnortoncmjw@outlook.com|UBKt4Wco1Q|M.C525_BAY.0.U.-Cv29HbLpga1twhmuvjUUrkj14xEX9HmUFGYm5Aweyy4g1vSwnq*H5LhmJnlW3b5RUebFjSVtycn0uVKh3e32s!ZWnS1fcrFJKIRJXobdBhga7ouSZ21qfyHdd1UCHoYtu1FY!mm1GKmkmu77qakQ9ezR5!BO59RcSjSEJla84Djf*m8NtyngsVTvs0*WFFrXOOK8Nlezh91s59LKuffkOnp8Djs60nNrENbcKWYAcRTNW2!NLE6YVttSA!9W!swFqIGxhwc9x*ZWG!NZCovIacukuYwEFeH853G2wc*o0SfZ*zXRPNb06wQIXWQTtOMoxUiQUdF7FUJDLhm6m6aPn!gnwHE3bROQHmq8klDL76!ApxM*GofqMSxH58PGPW4qxVi8k2u6CtMbmtMZ1jeXcnxPnBb0ap2YCoCUIRUQ7kuD|9e5f94bc-e8a4-4e73-b8be-63364c29d753" xr:uid="{C107134A-68B5-47D9-8D49-3393750BFE42}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>